<commit_message>
Flag cytotoxic cancer drugs as less relevant
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0172aZyF91urYrmsEU7SxkRE
</commit_message>
<xml_diff>
--- a/research/SurTrac_Drug_Company_Scoring.xlsx
+++ b/research/SurTrac_Drug_Company_Scoring.xlsx
@@ -54,7 +54,7 @@
     <t xml:space="preserve">Company-level check: only 29% of the earlier EU country listings (1,063 of 3,660) are backed by the company's own authorisation. Glenmark loses azacitidine and plerixafor (no own Tier 1 authorisation) and drops from 6th to 11th. Alembic loses carboprost.</t>
   </si>
   <si>
-    <t xml:space="preserve">Watch-outs on Lead drugs: 20 are cytotoxics (pitch must fit hazardous-drug handling rules), 31 are powders needing reconstitution, and 13 are already prefilled syringes (pitch as a safety upgrade).</t>
+    <t xml:space="preserve">Watch-outs on Lead drugs: 20 are cytotoxic cancer drugs (flagged as less relevant: usually pharmacy-prepared with closed transfer devices), 31 are powders needing reconstitution, and 13 are already prefilled syringes (pitch as a safety upgrade).</t>
   </si>
   <si>
     <t xml:space="preserve">Deprioritise Lupin, Strides and Alembic (1–3 Lead drugs). Their portfolios in this list are low-priced or lack their own authorisation in a Tier 1 market.</t>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Powder – check reconstitution volume</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution; Crowded (7 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution; Crowded (7 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Differentiation in crowded generic market</t>
@@ -306,7 +306,7 @@
     <t xml:space="preserve">Vial, Prefilled syringe</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution; Crowded (10 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution; Crowded (10 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Amoxicillin</t>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">UK-NI, DE, FR, NL, BE, CA</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant</t>
   </si>
   <si>
     <t xml:space="preserve">Safety-device mandate compliance</t>
@@ -399,7 +399,7 @@
     <t xml:space="preserve">Oncology – breast cancer, lymphomas, sarcomas, leukaemia</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Crowded (4 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Crowded (4 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">UK-NI, DE, FR, CA</t>
@@ -429,7 +429,7 @@
     <t xml:space="preserve">UK, UK-NI, DE, FR, NL, BE, CA</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution; Crowded (5 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution; Crowded (5 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Eribulin</t>
@@ -519,7 +519,7 @@
     <t xml:space="preserve">Oncology – stem-cell transplant conditioning; breast, ovarian &amp; bladder cancers</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution</t>
   </si>
   <si>
     <t xml:space="preserve">Crowded (3 cos)</t>
@@ -825,7 +825,7 @@
     <t xml:space="preserve">Oncology – Hodgkin lymphoma, testicular &amp; squamous cell cancers</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution; Crowded (3 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution; Crowded (3 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Baclofen</t>
@@ -1095,7 +1095,7 @@
     <t xml:space="preserve">DE, FR, BE</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Crowded (3 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Crowded (3 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Mesna</t>
@@ -1155,10 +1155,10 @@
     <t xml:space="preserve">Vaccines – childhood measles immunisation</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic; Crowded (10 cos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cytotoxic; Reconstitution; Crowded (4 cos)</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Crowded (10 cos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant; Reconstitution; Crowded (4 cos)</t>
   </si>
   <si>
     <t xml:space="preserve">Phenylephrine</t>
@@ -5274,7 +5274,7 @@
     <t xml:space="preserve">Watch-outs (not exclusions)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytotoxic (pharmacy-compounded under hazardous-drug rules; closed-system transfer devices compete); Reconstitution (powder – may need a transfer device or second syringe); Crowded (≥3 target companies make it – a differentiation argument for SurTrac); Prefilled only (pitch as safety upgrade). "Fits 1–10 mL syringe" reads fill volume from strength/packaging text; powders are judged by reconstitution volume, not vial size.</t>
+    <t xml:space="preserve">Cancer drug (cytotoxic) – less relevant: usually prepared in hospital pharmacies with closed-system transfer devices rather than standard syringes; kept in the ranking but flagged; Reconstitution (powder – may need a transfer device or second syringe); Crowded (≥3 target companies make it – a differentiation argument for SurTrac); Prefilled only (pitch as safety upgrade). "Fits 1–10 mL syringe" reads fill volume from strength/packaging text; powders are judged by reconstitution volume, not vial size.</t>
   </si>
   <si>
     <t xml:space="preserve">Company group entities matched</t>
@@ -6673,7 +6673,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
         <v>19</v>
       </c>
@@ -6759,7 +6759,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12"/>
       <c r="B7" s="20" t="s">
         <v>73</v>
@@ -7093,7 +7093,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>21</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12"/>
       <c r="B16" s="20" t="s">
         <v>73</v>
@@ -7347,7 +7347,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12"/>
       <c r="B21" s="12" t="s">
         <v>103</v>
@@ -7513,7 +7513,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
         <v>23</v>
       </c>
@@ -7557,7 +7557,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12"/>
       <c r="B26" s="20" t="s">
         <v>73</v>
@@ -7933,7 +7933,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
         <v>25</v>
       </c>
@@ -7977,7 +7977,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12"/>
       <c r="B36" s="20" t="s">
         <v>73</v>
@@ -8355,7 +8355,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
         <v>27</v>
       </c>
@@ -8441,7 +8441,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12"/>
       <c r="B47" s="20" t="s">
         <v>73</v>
@@ -8609,7 +8609,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12"/>
       <c r="B51" s="12" t="s">
         <v>103</v>
@@ -8775,7 +8775,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13" t="s">
         <v>29</v>
       </c>
@@ -8945,7 +8945,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12"/>
       <c r="B59" s="20" t="s">
         <v>73</v>
@@ -9909,7 +9909,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="13" t="s">
         <v>35</v>
       </c>
@@ -10201,7 +10201,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="13" t="s">
         <v>37</v>
       </c>
@@ -10701,7 +10701,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="12"/>
       <c r="B101" s="20" t="s">
         <v>73</v>
@@ -11449,7 +11449,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="12"/>
       <c r="B119" s="20" t="s">
         <v>73</v>
@@ -12788,7 +12788,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
         <v>23</v>
       </c>
@@ -12844,7 +12844,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
         <v>23</v>
       </c>
@@ -13178,7 +13178,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
         <v>23</v>
       </c>
@@ -13290,7 +13290,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
         <v>23</v>
       </c>
@@ -13510,7 +13510,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
         <v>23</v>
       </c>
@@ -13620,7 +13620,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
         <v>23</v>
       </c>
@@ -15052,7 +15052,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
         <v>23</v>
       </c>
@@ -16232,7 +16232,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
         <v>31</v>
       </c>
@@ -16290,7 +16290,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
         <v>31</v>
       </c>
@@ -16348,7 +16348,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
         <v>31</v>
       </c>
@@ -16518,7 +16518,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
         <v>31</v>
       </c>
@@ -16808,7 +16808,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
         <v>31</v>
       </c>
@@ -17038,7 +17038,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
         <v>25</v>
       </c>
@@ -17094,7 +17094,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
         <v>25</v>
       </c>
@@ -17486,7 +17486,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
         <v>25</v>
       </c>
@@ -17598,7 +17598,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="12" t="s">
         <v>25</v>
       </c>
@@ -18378,7 +18378,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="12" t="s">
         <v>21</v>
       </c>
@@ -18434,7 +18434,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="12" t="s">
         <v>21</v>
       </c>
@@ -18658,7 +18658,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="12" t="s">
         <v>21</v>
       </c>
@@ -18714,7 +18714,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="12" t="s">
         <v>21</v>
       </c>
@@ -18770,7 +18770,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="12" t="s">
         <v>21</v>
       </c>
@@ -19602,7 +19602,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="12" t="s">
         <v>39</v>
       </c>
@@ -19658,7 +19658,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="12" t="s">
         <v>39</v>
       </c>
@@ -19714,7 +19714,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="12" t="s">
         <v>39</v>
       </c>
@@ -19830,7 +19830,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="12" t="s">
         <v>27</v>
       </c>
@@ -19942,7 +19942,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="12" t="s">
         <v>27</v>
       </c>
@@ -20166,7 +20166,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="12" t="s">
         <v>27</v>
       </c>
@@ -21054,7 +21054,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="12" t="s">
         <v>19</v>
       </c>
@@ -21166,7 +21166,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="12" t="s">
         <v>19</v>
       </c>
@@ -21556,7 +21556,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="12" t="s">
         <v>19</v>
       </c>
@@ -22112,7 +22112,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="12" t="s">
         <v>19</v>
       </c>
@@ -22168,7 +22168,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="12" t="s">
         <v>19</v>
       </c>
@@ -22224,7 +22224,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="12" t="s">
         <v>19</v>
       </c>
@@ -22280,7 +22280,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="12" t="s">
         <v>19</v>
       </c>
@@ -22390,7 +22390,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="12" t="s">
         <v>19</v>
       </c>
@@ -23058,7 +23058,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
         <v>19</v>
       </c>
@@ -23114,7 +23114,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
         <v>19</v>
       </c>
@@ -25470,7 +25470,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="12" t="s">
         <v>35</v>
       </c>
@@ -27358,7 +27358,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="12" t="s">
         <v>29</v>
       </c>
@@ -27526,7 +27526,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="12" t="s">
         <v>29</v>
       </c>
@@ -27582,7 +27582,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="277" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="12" t="s">
         <v>29</v>
       </c>
@@ -28748,7 +28748,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="298" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="12" t="s">
         <v>45</v>
       </c>
@@ -30016,7 +30016,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="321" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="12" t="s">
         <v>37</v>
       </c>
@@ -62487,7 +62487,7 @@
         <v>1745</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="s">
         <v>1746</v>
       </c>

</xml_diff>